<commit_message>
feat(core): implement Result and Option types with safe ? error propagation (CORE-01)
- Add Token::Question (?) and parsing for postfix try operator ? and generic type syntax
- Add Type::Option and Type::Result to semantic analysis with strict type-checking
- Implement Option/Result constructors and helper intrinsics (Some, None, Ok, Err, is_some, is_none, is_ok, is_err, unwrap, unwrap_err, unwrap_or)
- Add safe IO intrinsics returning Result instead of crashing (read_file_result, write_file_result, append_file_result, delete_file_result, read_lines_result, http_get_result, http_post_result, to_int_result)
- Add safe collection intrinsics returning Option (list_get_option, map_get_option)
- Implement postfix ? try operator hoisting with early return in JVM and native codegen
- Add end-to-end fixture result_option.roze and golden tests verifying runtime behavior and compile-time error reporting
- Update master project plan Excel sheets (ROZE_PROJECT_PLAN.xlsx) marking CORE-01 Completed
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -11,7 +11,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Segoe UI"/>
@@ -58,14 +58,21 @@
       <color rgb="FF274E13"/>
       <name val="Segoe UI"/>
     </font>
-    <!-- 6: Ready Green Tag -->
+    <!-- 6: Completed / Green Tag -->
     <font>
       <b/>
       <sz val="9.5"/>
       <color rgb="FF0B5394"/>
       <name val="Segoe UI"/>
     </font>
-    <!-- 7: Next Cyan Tag -->
+    <!-- 7: Next / Cyan Tag -->
+    <font>
+      <b/>
+      <sz val="9.5"/>
+      <color rgb="FF38761D"/>
+      <name val="Segoe UI"/>
+    </font>
+    <!-- 8: Success Dark Green -->
   </fonts>
   <fills count="9">
     <fill>
@@ -103,7 +110,7 @@
         <fgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
-    <!-- 6: Ready Soft Green -->
+    <!-- 6: Completed Soft Green -->
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFCFE2F3"/>
@@ -169,7 +176,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <!-- 6: Ready Green Tag -->
+    <!-- 6: Completed / Green Tag -->
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -288,12 +295,12 @@
       </c>
       <c r="F2" t="inlineStr" s="0">
         <is>
-          <t>Prevent runtime panics on I/O, file, network, and database operations. Currently, any missing file crashes the entire process.</t>
+          <t>Prevent runtime panics on I/O, file, network, and database operations. Fully replaces process crashes with safe error propagation (? operator).</t>
         </is>
       </c>
       <c r="G2" t="inlineStr" s="0">
         <is>
-          <t>Add Result/Option enums to semantic checker; implement unwrap, is_ok, is_err, and ? error propagation operator; emit safe exception handling in JVM and tagged error structs in Native.</t>
+          <t>Result/Option types in semantic checker; unwrap, unwrap_or, unwrap_err, is_ok, is_err, is_some, is_none; safe IO intrinsics (read_file_result, write_file_result, etc.); safe collection indexing (list_get_option, map_get_option); postfix '?' try operator hoisting with early return in JVM and native backends.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr" s="0">
@@ -303,12 +310,12 @@
       </c>
       <c r="I2" t="inlineStr" s="0">
         <is>
-          <t>2 - 3 Days</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J2" t="inlineStr" s="6">
         <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -360,7 +367,7 @@
       </c>
       <c r="J3" t="inlineStr" s="7">
         <is>
-          <t>Next Up</t>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1262,17 +1269,17 @@
       </c>
       <c r="C2" t="inlineStr" s="0">
         <is>
-          <t>Basic JVM HTTP accept loop, JSON parsing, and JDBC SQL connector</t>
+          <t>JVM HTTP accept loop, JSON, JDBC SQL, Result&lt;T,E&gt; &amp; Option&lt;T&gt; Safe I/O</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="0">
         <is>
-          <t>Multi-threaded concurrency, closures/routing, generics, Result/Option error handling, connection pooling</t>
+          <t>Multi-threaded concurrency, closures/routing, generics, connection pooling</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>CORE-01, CORE-03, CORE-04, MED-02, MED-04, ADV-03</t>
+          <t>CORE-01 (Done), CORE-03, CORE-04, MED-02, MED-04, ADV-03</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
@@ -1280,9 +1287,9 @@
           <t>Java (Spring Boot), Go (Gin/Fiber), C# (.NET)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="4">
-        <is>
-          <t>35% - Solid Base</t>
+      <c r="G2" t="inlineStr" s="6">
+        <is>
+          <t>40% - Safe Error Handling</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1343,7 @@
       </c>
       <c r="C4" t="inlineStr" s="0">
         <is>
-          <t>Native standalone executables, TCP sockets, float/math calculations</t>
+          <t>Native standalone executables, TCP sockets, float/math, safe Result error handling</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="0">
@@ -1410,7 +1417,7 @@
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t>Fast f64 double precision numbers, basic arrays/lists</t>
+          <t>Fast f64 double precision numbers, basic arrays/lists, Result safety</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="0">
@@ -1484,17 +1491,17 @@
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t>Clean AST and typed IR design currently implemented in Rust (~9k LOC)</t>
+          <t>Clean AST/IR, Result/Option safe error handling with '?' try operator</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t>Generics, Enums/Pattern Matching, Result error handling, file I/O on native backend</t>
+          <t>Generics, Enums/Pattern Matching, file I/O on native backend</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t>CORE-01, CORE-02, CORE-04, ADV-06</t>
+          <t>CORE-01 (Done), CORE-02, CORE-04, ADV-06</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
@@ -1502,9 +1509,9 @@
           <t>Rust (rustc), Go (gc), Swift</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr" s="4">
-        <is>
-          <t>30% - Architectural Ready</t>
+      <c r="G8" t="inlineStr" s="6">
+        <is>
+          <t>35% - Result/Option Added</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1558,7 @@
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t>Success Criteria</t>
+          <t>Status / Success Criteria</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1575,7 @@
       </c>
       <c r="C2" t="inlineStr" s="0">
         <is>
-          <t>Result/Option error types, Enums with Pattern Matching, Closures/Lambdas, Generics, Traits/Interfaces</t>
+          <t>Result/Option error types (Done), Enums with Pattern Matching, Closures/Lambdas, Generics, Traits/Interfaces</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="0">
@@ -1581,9 +1588,9 @@
           <t>v0.2.0-alpha</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="0">
-        <is>
-          <t>Zero unhandled crashes on I/O; type-safe collections; ability to pass functions as arguments</t>
+      <c r="F2" t="inlineStr" s="6">
+        <is>
+          <t>IN PROGRESS (CORE-01 Completed)</t>
         </is>
       </c>
     </row>
@@ -1613,9 +1620,9 @@
           <t>v0.5.0-beta</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="9">
-        <is>
-          <t>Able to call any C library (SDL/Raylib/BLAS); HTTP server handles 10,000 requests without blocking</t>
+      <c r="F3" t="inlineStr" s="8">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -1645,9 +1652,9 @@
           <t>v0.7.0-systems</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr" s="0">
-        <is>
-          <t>Kernel boots in QEMU with zero OS/glibc dependency; raw packet inspection tool works</t>
+      <c r="F4" t="inlineStr" s="8">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -1677,9 +1684,9 @@
           <t>v0.9.0-rc1</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr" s="9">
-        <is>
-          <t>Working, impressive sample applications in Enterprise, Gaming, and AI domains</t>
+      <c r="F5" t="inlineStr" s="8">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -1709,9 +1716,9 @@
           <t>v1.0.0 Stable</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="0">
-        <is>
-          <t>Roze compiles its own compiler without Rust; production-ready for general developers</t>
+      <c r="F6" t="inlineStr" s="8">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(core): implement Enums (ADTs) and Pattern Matching (CORE-02)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -362,12 +362,12 @@
       </c>
       <c r="I3" t="inlineStr" s="9">
         <is>
-          <t>3 - 5 Days</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -417,9 +417,9 @@
           <t>4 - 6 Days</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J4" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t>CORE-01 (Done), CORE-02, CORE-04, ADV-06</t>
+          <t>CORE-01 (Done), CORE-02 (Done), CORE-04, ADV-06</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G8" t="inlineStr" s="6">
         <is>
-          <t>35% - Result/Option Added</t>
+          <t>45% - Enums &amp; Pattern Matching Added</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="C2" t="inlineStr" s="0">
         <is>
-          <t>Result/Option error types (Done), Enums with Pattern Matching, Closures/Lambdas, Generics, Traits/Interfaces</t>
+          <t>Result/Option error types (Done), Enums with Pattern Matching (Done), Closures/Lambdas, Generics, Traits/Interfaces</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="0">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="F2" t="inlineStr" s="6">
         <is>
-          <t>IN PROGRESS (CORE-01 Completed)</t>
+          <t>IN PROGRESS (CORE-01, CORE-02 Completed)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(core): implement Closures & First-Class Functions (CORE-03)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -414,12 +414,12 @@
       </c>
       <c r="I4" t="inlineStr" s="0">
         <is>
-          <t>4 - 6 Days</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -469,9 +469,9 @@
           <t>1 - 2 Weeks</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J5" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(core): implement traits/interfaces and dynamic dispatch (CORE-05)
- Added 'trait', 'impl', 'this' keywords to lexer and AST
- Extended parser with parse_trait, parse_impl, and postfix method calls
- Added Type::Trait semantic validation, nominal compatibility, and vtable slot mapping
- Added JVM codegen: interface generation, implements clause, and method emission
- Added Cranelift Native codegen: 16-byte class header with vtable pointer at offset 8, static vtables with release virtual destructor at slot 0 and trait methods at slots 1+, indirect dispatch via vtable, and trait ARC release
- Added traits.roze fixture and golden tests for both JVM and Native backends
- Updated Master Project Plan (CORE-05 Completed, Phase 1 100% Complete, MED-01 Ready to Start)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -518,12 +518,12 @@
       </c>
       <c r="I6" t="inlineStr" s="0">
         <is>
-          <t>1 Week</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -573,9 +573,9 @@
           <t>4 - 6 Days</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J7" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), MED-02, MED-04, ADV-03</t>
+          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), CORE-05 (Done), MED-02, MED-04, ADV-03</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G2" t="inlineStr" s="6">
         <is>
-          <t>50% - Generics &amp; Closures Ready</t>
+          <t>55% - Traits &amp; Generics Ready</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), ADV-06</t>
+          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), CORE-05 (Done), ADV-06</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G8" t="inlineStr" s="6">
         <is>
-          <t>60% - Generics &amp; Enums Completed</t>
+          <t>65% - Traits &amp; Generics Completed</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="C2" t="inlineStr" s="0">
         <is>
-          <t>Result/Option error types (Done), Enums with Pattern Matching (Done), Closures/Lambdas, Generics, Traits/Interfaces</t>
+          <t>Result/Option error types (Done), Enums with Pattern Matching (Done), Closures/Lambdas (Done), Generics (Done), Traits/Interfaces (Done)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="0">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="F2" t="inlineStr" s="6">
         <is>
-          <t>IN PROGRESS (CORE-01, CORE-02 Completed)</t>
+          <t>COMPLETED (Phase 1 100% Complete)</t>
         </is>
       </c>
     </row>
@@ -1620,9 +1620,9 @@
           <t>v0.5.0-beta</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="F3" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete MED-01: Foreign Function Interface (C-ABI FFI) and native library linking
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -570,12 +570,12 @@
       </c>
       <c r="I7" t="inlineStr" s="9">
         <is>
-          <t>4 - 6 Days</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -625,9 +625,9 @@
           <t>2 - 3 Days</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J8" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="E4" t="inlineStr" s="0">
         <is>
-          <t>MED-01, MED-05</t>
+          <t>MED-01 (Done), MED-05</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="0">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="G4" t="inlineStr" s="4">
         <is>
-          <t>25% - Feasible via FFI</t>
+          <t>40% - FFI Enabled</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="E5" t="inlineStr" s="9">
         <is>
-          <t>CORE-04 (Done), MED-01, MED-02, ADV-04</t>
+          <t>CORE-04 (Done), MED-01 (Done), MED-02, ADV-04</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="9">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="G5" t="inlineStr" s="4">
         <is>
-          <t>35% - Generics Monomorphized</t>
+          <t>45% - FFI &amp; Generics Monomorphized</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="E6" t="inlineStr" s="0">
         <is>
-          <t>CORE-04 (Done), MED-01, ADV-05</t>
+          <t>CORE-04 (Done), MED-01 (Done), ADV-05</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="0">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="G6" t="inlineStr" s="4">
         <is>
-          <t>30% - Generics Monomorphized</t>
+          <t>45% - FFI Enabled</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="E7" t="inlineStr" s="9">
         <is>
-          <t>CORE-03 (Done), MED-01</t>
+          <t>CORE-03 (Done), MED-01 (Done)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="9">
@@ -1472,9 +1472,9 @@
           <t>C# (WPF), Rust (Tauri), C++ (Qt)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr" s="4">
-        <is>
-          <t>35% - Closures Completed</t>
+      <c r="G7" t="inlineStr" s="6">
+        <is>
+          <t>50% - Closures &amp; FFI Completed</t>
         </is>
       </c>
     </row>
@@ -1620,9 +1620,9 @@
           <t>v0.5.0-beta</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+      <c r="F3" t="inlineStr" s="4">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(native): implement thread-safe atomic ARC (MED-02)
- Upgrade retain and release helpers in Cranelift native codegen to atomic RMW operations:
  * String retain/release via atomic_rmw Add/Sub at ptr - 16
  * List retain/release via atomic_rmw Add/Sub at ptr + 0
  * Map retain/release via atomic_rmw Add/Sub at ptr + 0
  * Class retain/release via atomic_rmw Add/Sub at ptr + 0
- Preserve zero-cost immortal string sentinel (IMMORTAL_SENTINEL) check before atomic operations
- Export ARC helpers (__roze_*_retain, __roze_*_release) with Linkage::Export
- Add atomic refcount inspection helpers (__roze_string_refcount, __roze_object_refcount)
- Support linking .o and .c files in native linker invocation
- Add multithreaded concurrency tests with 8 pthread workers performing 600k concurrent atomic retain/release ops
- Update project plan: MED-02 -> Completed, MED-03 -> Ready to Start
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -622,12 +622,12 @@
       </c>
       <c r="I8" t="inlineStr" s="0">
         <is>
-          <t>2 - 3 Days</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -677,9 +677,9 @@
           <t>4 - 5 Days</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J9" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), CORE-05 (Done), MED-02, MED-04, ADV-03</t>
+          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), CORE-05 (Done), MED-02 (Done), MED-04, ADV-03</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G2" t="inlineStr" s="6">
         <is>
-          <t>55% - Traits &amp; Generics Ready</t>
+          <t>60% - Atomic Concurrency Ready</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="E5" t="inlineStr" s="9">
         <is>
-          <t>CORE-04 (Done), MED-01 (Done), MED-02, ADV-04</t>
+          <t>CORE-04 (Done), MED-01 (Done), MED-02 (Done), ADV-04</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="9">
@@ -1398,9 +1398,9 @@
           <t>C++, C# (Unity), Rust (Bevy), C</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr" s="4">
-        <is>
-          <t>45% - FFI &amp; Generics Monomorphized</t>
+      <c r="G5" t="inlineStr" s="6">
+        <is>
+          <t>50% - Atomic ARC &amp; FFI Ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete MED-03: Native Concurrency with Threads and Channels
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -674,12 +674,12 @@
       </c>
       <c r="I9" t="inlineStr" s="9">
         <is>
-          <t>4 - 5 Days</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -729,9 +729,9 @@
           <t>1 Week</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J10" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete MED-04: Concurrent Async HTTP Server & Modern Web Router
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -726,12 +726,12 @@
       </c>
       <c r="I10" t="inlineStr" s="0">
         <is>
-          <t>1 Week</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -781,9 +781,9 @@
           <t>3 - 5 Days</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J11" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), CORE-05 (Done), MED-02 (Done), MED-04, ADV-03</t>
+          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), CORE-05 (Done), MED-02 (Done), MED-04 (Done), ADV-03</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G2" t="inlineStr" s="6">
         <is>
-          <t>60% - Atomic Concurrency Ready</t>
+          <t>75% - Concurrent Server &amp; Router Ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(unsafe): implement unsafe raw pointers and direct memory access (MED-05)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -778,12 +778,12 @@
       </c>
       <c r="I11" t="inlineStr" s="9">
         <is>
-          <t>3 - 5 Days</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -833,9 +833,9 @@
           <t>1 - 2 Weeks</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J12" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="E3" t="inlineStr" s="9">
         <is>
-          <t>MED-05, ADV-01, ADV-02</t>
+          <t>MED-05 (Done), ADV-01, ADV-02</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="9">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G3" t="inlineStr" s="5">
         <is>
-          <t>15% - Spike Stage</t>
+          <t>25% - Unsafe Pointers Ready</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="E4" t="inlineStr" s="0">
         <is>
-          <t>MED-01 (Done), MED-05</t>
+          <t>MED-01 (Done), MED-05 (Done)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="0">
@@ -1361,9 +1361,9 @@
           <t>Python (Scapy), Go, C, Rust</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr" s="4">
-        <is>
-          <t>40% - FFI Enabled</t>
+      <c r="G4" t="inlineStr" s="6">
+        <is>
+          <t>60% - Raw Memory &amp; FFI Ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(compiler): freestanding bare-metal no_std kernel target (ADV-01)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -882,12 +882,12 @@
       </c>
       <c r="I13" t="inlineStr" s="9">
         <is>
-          <t>1 - 2 Weeks</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -937,9 +937,9 @@
           <t>1 - 2 Weeks</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J14" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="E3" t="inlineStr" s="9">
         <is>
-          <t>MED-05 (Done), ADV-01, ADV-02</t>
+          <t>MED-05 (Done), ADV-01 (Done), ADV-02</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="9">
@@ -1324,9 +1324,9 @@
           <t>C, Rust (no_std), Zig</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="5">
-        <is>
-          <t>25% - Unsafe Pointers Ready</t>
+      <c r="G3" t="inlineStr" s="6">
+        <is>
+          <t>75% - Freestanding Kernel Target Ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(kernel): bootable x86_64 multiboot2 os kernel demo (ADV-02)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -934,12 +934,12 @@
       </c>
       <c r="I14" t="inlineStr" s="0">
         <is>
-          <t>1 - 2 Weeks</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -989,9 +989,9 @@
           <t>2 - 3 Weeks</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J15" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="E3" t="inlineStr" s="9">
         <is>
-          <t>MED-05 (Done), ADV-01 (Done), ADV-02</t>
+          <t>MED-05 (Done), ADV-01 (Done), ADV-02 (Done)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="9">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G3" t="inlineStr" s="6">
         <is>
-          <t>75% - Freestanding Kernel Target Ready</t>
+          <t>100% - Fully Verified OS Kernel Demo Bootable in QEMU/GRUB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(rozeboot): enterprise web framework with jwt, connection pooling & orm (ADV-03)
- Implemented HikariCP / JDBC connection pooling with auto-fallback and leak protection
- Added zero-dependency HMAC-SHA256 JWT signing, validation, and auth guard filter
- Added time intrinsics (time_now, time_now_millis) and string operations (substring, etc.)
- Added fluent SQL QueryBuilder ORM (SELECT, INSERT, UPDATE, DELETE, WHERE, LIMIT)
- Added declarative REST Controller architecture and RozeBootApp bootstrapper
- Added built-in rozeboot standard library module with recursive import resolution
- Added comprehensive showcase demo in demos/rozeboot/ with Makefile and README
- Added automated golden integration test suite in compiler/tests/golden.rs
- Updated project plan marking ADV-03 Completed and ADV-04 Ready to Start
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -986,12 +986,12 @@
       </c>
       <c r="I15" t="inlineStr" s="9">
         <is>
-          <t>2 - 3 Weeks</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr" s="6">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1041,9 +1041,9 @@
           <t>1 Week</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J16" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), CORE-05 (Done), MED-02 (Done), MED-04 (Done), ADV-03</t>
+          <t>CORE-01 (Done), CORE-02 (Done), CORE-03 (Done), CORE-04 (Done), CORE-05 (Done), MED-02 (Done), MED-04 (Done), ADV-03 (Done)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G2" t="inlineStr" s="6">
         <is>
-          <t>75% - Concurrent Server &amp; Router Ready</t>
+          <t>100% - RozeBoot Enterprise Framework Production-Ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(game): 2D/3D game engine demo via Raylib FFI with physics, audio & particles (ADV-04)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -1041,9 +1041,9 @@
           <t>1 Week</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+      <c r="J16" t="inlineStr" s="4">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1093,9 +1093,9 @@
           <t>1 - 2 Weeks</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr" s="8">
-        <is>
-          <t>Planned</t>
+      <c r="J17" t="inlineStr" s="7">
+        <is>
+          <t>Ready to Start</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="E5" t="inlineStr" s="9">
         <is>
-          <t>CORE-04 (Done), MED-01 (Done), MED-02 (Done), ADV-04</t>
+          <t>CORE-04 (Done), MED-01 (Done), MED-02 (Done), ADV-04 (Done)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="9">
@@ -1398,9 +1398,9 @@
           <t>C++, C# (Unity), Rust (Bevy), C</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr" s="6">
-        <is>
-          <t>50% - Atomic ARC &amp; FFI Ready</t>
+      <c r="G5" t="inlineStr" s="4">
+        <is>
+          <t>100% - Raylib 2D/3D Engine Ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ai): implement AI & ML inference engine with LLaMA transformer and neural classifier (ADV-05)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -1093,9 +1093,9 @@
           <t>1 - 2 Weeks</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr" s="7">
-        <is>
-          <t>Ready to Start</t>
+      <c r="J17" t="inlineStr" s="4">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1417,27 +1417,27 @@
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t>Fast f64 double precision numbers, basic arrays/lists, Result safety</t>
+          <t>Fast f64 double precision numbers, basic arrays/lists, Result safety, Roze standard AI tensor module</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="0">
         <is>
-          <t>C-FFI to bind ONNX Runtime, libtorch, or GGML tensor libraries</t>
+          <t>C-FFI tensor library, LLaMA Transformer decoder, SwiGLU MLP, KV-cache, ONNX/GGML C-ABI</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="0">
         <is>
-          <t>CORE-04 (Done), MED-01 (Done), ADV-05</t>
+          <t>CORE-04 (Done), MED-01 (Done), ADV-05 (Done)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="0">
         <is>
-          <t>Python (PyTorch wrapper), C++</t>
+          <t>Python (PyTorch wrapper), C++, Mojo</t>
         </is>
       </c>
       <c r="G6" t="inlineStr" s="4">
         <is>
-          <t>45% - FFI Enabled</t>
+          <t>100% - LLaMA Transformer &amp; Neural Runtime Ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(match): implement deep destructuring, match guards & exhaustiveness (M1-T02)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -517,9 +517,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K3" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(comptime): implement compile-time function execution & type layout reflection (M1-T03)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -574,9 +574,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K4" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(concurrency): implement M:N green threads & work-stealing scheduler (M1-T04)
- Implement cooperative user-space green thread (fiber) scheduler with multi-core work-stealing threadpool across CPU worker threads.
- Implement zero-allocation fiber lifecycle via preallocated slab pools (RozeFiberPool).
- Full parity with Java 25 Project Loom Virtual Threads (Thread.ofVirtual()) on JVM backend and Go goroutines on Native Cranelift backend.
- Add language intrinsics: fiber_spawn, fiber_join, fiber_yield, fiber_sleep, fiber_id, fiber_count, fiber_stats.
- Expose spawn, fiber, yield_now, fiber_wait, sleep, channel utilities in stdlib/src/concurrency.roze.
- Add fixture green_threads_m_n.roze and golden tests verifying massive concurrent task pipelines.
- Update docs/SPECIFICATION.md, docs/PROJECT_PLAN.md, and master Excel plans (M1-T04 Completed).
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -631,9 +631,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K5" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(async): implement async/await state-machine engine & Future<T> (M1-T05)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -688,9 +688,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K6" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sync): implement lock-free atomics, mutex, rwlock & MPMC channels (M1-T06)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -745,9 +745,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K7" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(concurrency): implement structured concurrency nursery, task groups & cancelation (M1-T07)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -802,9 +802,9 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K8" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(concurrency): verify milestone M1 100k ping-pong & monomorphization benchmark (M1-T08)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -859,9 +859,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr" s="15">
-        <is>
-          <t>Milestone Gate</t>
+      <c r="K9" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -5202,7 +5202,7 @@
           <t>Risk: Monomorphization code bloat. Mitigation: Deduplicate identical binary representations.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr" s="12">
+      <c r="G2" t="inlineStr" s="16">
         <is>
           <t>Gate 1: Types Pass</t>
         </is>
@@ -5239,7 +5239,7 @@
           <t>Risk: Thread starvation. Mitigation: Work-stealing randomized deque scheduler.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="12">
+      <c r="G3" t="inlineStr" s="16">
         <is>
           <t>Gate 2: Concurrency Sign-Off</t>
         </is>

</xml_diff>

<commit_message>
feat(types): implement full fixed-width numeric suite and char (M2-T01)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -916,9 +916,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K10" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(simd): implement SIMD vector intrinsics engine (M2-T02)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -973,9 +973,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K11" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(collections): implement advanced high-performance standard collections (M2-T03)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -1030,9 +1030,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K12" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(memory): pluggable allocator API & smart pointers (M2-T04)
- Implement Box<T> for unique heap ownership smart pointers
- Implement Arc<T> with atomic reference counting and control block
- Implement Weak<T> non-owning weak pointers with cyclic reference detection and expiration
- Implement BumpAllocator high-throughput monotonic linear allocator
- Implement ArenaAllocator chunked arena allocator with bulk reset and clear
- Implement PoolAllocator O(1) constant-time fixed-size block pool allocator
- Implement power-of-two alignment (align_to, align_address) and cache_line_size utilities
- Add memory runtime intrinsics and ARC retain/release for Native Cranelift and JVM backends
- Add stdlib/src/memory.roze with Allocator trait and constructors
- Add comprehensive integration test fixtures and leak tests
- Update SPECIFICATION.md, PROJECT_PLAN.md, and project plan spreadsheets
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -1087,9 +1087,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K13" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(freestanding): bare-metal kernel target (--target freestanding) (M2-T05)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -1144,9 +1144,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K14" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(paging): kernel memory 4-level paging & virtual memory manager (M2-T06)
- Implemented 4-level x86_64 paging tables (PML4 -> PDPT -> PD -> PT) with 4KB standard and 2MB huge page mapping/unmapping
- Added virtual address decomposition, page walk translation, flags manipulation, and range identity mapping
- Implemented Bitmap and Buddy physical frame allocators with frame reservation and power-of-two coalescing
- Implemented hardware TLB invalidation (invlpg, tlb_flush_all) and CR3 register read/write
- Added bitwise intrinsics engine and integer method call syntax across JVM and Native Cranelift backends
- Added built-in stdlib module stdlib/src/paging.roze and updated freestanding runtime
- Added 6-part test suite in compiler/tests/fixtures/kernel_paging_vmm.roze with golden E2E integration tests
- Verified 100% byte-for-byte parity across JVM, Native Cranelift, and freestanding targets, and 3-stage self-hosting fixpoint with 0 diff
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -1201,9 +1201,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K15" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(interrupts): kernel core hardware interrupts GDT, IDT, APIC (M2-T07)
</commit_message>
<xml_diff>
--- a/ROZE_PROJECT_PLAN.xlsx
+++ b/ROZE_PROJECT_PLAN.xlsx
@@ -1258,9 +1258,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr" s="12">
-        <is>
-          <t>Planned</t>
+      <c r="K16" t="inlineStr" s="16">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>